<commit_message>
Update index rows B and B-6 with reclassified impairment figures
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/분석_인덱스.xlsx
+++ b/분석_인덱스.xlsx
@@ -1329,7 +1329,7 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>188건 전부 수집·검토. 분류 45건, 상태 21건, 금액 8건이 원자료와 다름. 그룹이 산 거래의 57%에서 인수 후 손상</t>
+          <t>188건 전부 수집·검토. 분류 45건, 상태 21건, 금액 10건이 원자료와 다름. 그룹이 산 거래 중 손상 여부를 판정할 수 있는 115건의 70%에서 인수 후 손상</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
@@ -1656,7 +1656,7 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>impairment</t>
+          <t>impairment_class (2026-11-01 재분류)</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
@@ -1671,12 +1671,12 @@
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>그룹이 산 139건 중 79건(57%) 손상, 53건 확인 안 됨. 로엔 1조 2,213억, Tapas·Radish 약 8,919억 전액 손상</t>
+          <t>그룹이 산 139건 중 판정 가능 115건(있음 81·없음 34)의 70% 손상. Kakao 81%, Naver 67%, CJ ENM 46%. 로엔 1조 2,213억, Tapas·Radish 약 8,919억 전액 손상</t>
         </is>
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>잠정 (확인 안 됨 53건, 생존 편향)</t>
+          <t>잠정 (식별 불가·미확인 15건 제외, 생존 편향)</t>
         </is>
       </c>
       <c r="J22" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Rename MA subtype labels by their basis, not 'raw data'
subtype was assigned in the 10-19 analysis from the comment, buyer and
seller fields; Capital IQ only provides 'Merger/Acquisition'. Labels are
now 'deal form (comment-based)' and 'deal form (filing-checked)'. Excel
columns are regrouped into Capital IQ raw fields, v4 sector (not checked
in collection), 10-19 comment-based fields and filing-checked fields.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/분석_인덱스.xlsx
+++ b/분석_인덱스.xlsx
@@ -1423,17 +1423,17 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>원자료 분류의 재판정</t>
+          <t>거래 형태 분류의 재판정</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>subtype_chk</t>
+          <t>subtype_chk (공시 확인)</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>subtype(원자료 기반)</t>
+          <t>subtype (10-19 설명란 판정)</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">

</xml_diff>